<commit_message>
Update Data_Teknis with Gambar 1 sites and update locations DB
</commit_message>
<xml_diff>
--- a/Template_Data_Teknis_Pentakom.xlsx
+++ b/Template_Data_Teknis_Pentakom.xlsx
@@ -36080,12 +36080,12 @@
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>-1.06316</t>
+          <t>-1,06316</t>
         </is>
       </c>
       <c r="I766" t="inlineStr">
         <is>
-          <t>120.493103</t>
+          <t>120,493103</t>
         </is>
       </c>
     </row>

</xml_diff>